<commit_message>
Agrega badge en la portada indicando si la familia trae pañales o pañitos, con soporte en la plantilla y el generador
</commit_message>
<xml_diff>
--- a/plantilla-invitados.xlsx
+++ b/plantilla-invitados.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>Familia</t>
   </si>
@@ -23,18 +23,27 @@
     <t>WhatsApp</t>
   </si>
   <si>
+    <t>Trae</t>
+  </si>
+  <si>
     <t>Familia Pérez</t>
   </si>
   <si>
     <t>573001234567</t>
   </si>
   <si>
+    <t>Pañales</t>
+  </si>
+  <si>
     <t>Familia Gómez</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
+    <t>Pañitos</t>
+  </si>
+  <si>
     <t>Ana y Luis</t>
   </si>
   <si>
@@ -53,13 +62,16 @@
     <t>3) Columna "WhatsApp" (opcional): número con indicativo de país sin "+" ni espacios (ej: 573001234567). Si lo llenas, el generador te crea un link listo para enviar por WhatsApp.</t>
   </si>
   <si>
-    <t>4) No cambies los nombres de las columnas ni el nombre de la hoja "Invitados".</t>
-  </si>
-  <si>
-    <t>5) Agrega todas las filas que necesites, una por familia/grupo.</t>
-  </si>
-  <si>
-    <t>6) Guarda el archivo y corre: node generar-invitaciones.js</t>
+    <t>4) Columna "Trae" (opcional): escribe "Pañales" o "Pañitos" para que la invitación de esa familia muestre ese distintivo en la portada. Si la dejas vacía, el generador alterna automáticamente entre las dos para repartir parejo.</t>
+  </si>
+  <si>
+    <t>5) No cambies los nombres de las columnas ni el nombre de la hoja "Invitados".</t>
+  </si>
+  <si>
+    <t>6) Agrega todas las filas que necesites, una por familia/grupo.</t>
+  </si>
+  <si>
+    <t>7) Guarda el archivo y corre: node generar-invitaciones.js</t>
   </si>
 </sst>
 </file>
@@ -445,15 +457,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -463,37 +476,49 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -505,7 +530,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
@@ -513,42 +538,47 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
El badge de la portada muestra ambas opciones (Pañales o Pañitos) para todos, en vez de asignar una por familia
</commit_message>
<xml_diff>
--- a/plantilla-invitados.xlsx
+++ b/plantilla-invitados.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>Familia</t>
   </si>
@@ -23,27 +23,18 @@
     <t>WhatsApp</t>
   </si>
   <si>
-    <t>Trae</t>
-  </si>
-  <si>
     <t>Familia Pérez</t>
   </si>
   <si>
     <t>573001234567</t>
   </si>
   <si>
-    <t>Pañales</t>
-  </si>
-  <si>
     <t>Familia Gómez</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Pañitos</t>
-  </si>
-  <si>
     <t>Ana y Luis</t>
   </si>
   <si>
@@ -62,16 +53,13 @@
     <t>3) Columna "WhatsApp" (opcional): número con indicativo de país sin "+" ni espacios (ej: 573001234567). Si lo llenas, el generador te crea un link listo para enviar por WhatsApp.</t>
   </si>
   <si>
-    <t>4) Columna "Trae" (opcional): escribe "Pañales" o "Pañitos" para que la invitación de esa familia muestre ese distintivo en la portada. Si la dejas vacía, el generador alterna automáticamente entre las dos para repartir parejo.</t>
-  </si>
-  <si>
-    <t>5) No cambies los nombres de las columnas ni el nombre de la hoja "Invitados".</t>
-  </si>
-  <si>
-    <t>6) Agrega todas las filas que necesites, una por familia/grupo.</t>
-  </si>
-  <si>
-    <t>7) Guarda el archivo y corre: node generar-invitaciones.js</t>
+    <t>4) No cambies los nombres de las columnas ni el nombre de la hoja "Invitados".</t>
+  </si>
+  <si>
+    <t>5) Agrega todas las filas que necesites, una por familia/grupo.</t>
+  </si>
+  <si>
+    <t>6) Guarda el archivo y corre: node generar-invitaciones.js</t>
   </si>
 </sst>
 </file>
@@ -457,16 +445,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -476,49 +463,37 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>4</v>
       </c>
       <c r="B2">
         <v>4</v>
       </c>
       <c r="C2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -530,7 +505,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
@@ -538,47 +513,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>